<commit_message>
ÚLTIMOS CAMBIOSgit add .!
</commit_message>
<xml_diff>
--- a/racheros/app/static/reportes/reporte_2_2025-12-01.xlsx
+++ b/racheros/app/static/reportes/reporte_2_2025-12-01.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H20"/>
+  <dimension ref="A2:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -519,7 +519,7 @@
     <row r="3">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Usuario: Jorge Isaac Ibañez Miranda | Periodo: 2025-12-01 al 2025-12-07</t>
+          <t>Usuario: Aldo Guzmán Martínez | Periodo: 2025-12-01 al 2025-12-07</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -584,7 +584,7 @@
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -601,7 +601,7 @@
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>2025-12-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -618,7 +618,7 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -652,7 +652,7 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -669,15 +669,49 @@
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Escuela / Tareas</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
           <t>2025-12-01</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Ir Al Gym</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>Escuela / Tareas</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Completado</t>
         </is>

</xml_diff>